<commit_message>
feat: added robustness checks and referee report
</commit_message>
<xml_diff>
--- a/report/Chris-Gabriel_Islam_Paper5_Replication_Log.xlsx
+++ b/report/Chris-Gabriel_Islam_Paper5_Replication_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Uni\Promotion\replication-game-kcl-2026\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355954EE-3528-4722-8208-9E32AD3B2CAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A24BF0-1617-4161-B425-347C286DE9FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Main" sheetId="1" r:id="rId1"/>
@@ -408,7 +408,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="105">
   <si>
     <t>Replication Game Metadata</t>
   </si>
@@ -653,9 +653,6 @@
     <t>Begin pasting in A25 and continue downward as needed. Do not type the report in the cells above.</t>
   </si>
   <si>
-    <t>[PASTE FULL REFEREE REPORT HERE]</t>
-  </si>
-  <si>
     <t>Figure 2</t>
   </si>
   <si>
@@ -693,6 +690,54 @@
   </si>
   <si>
     <t>Values in Figure are the same, formatting differs a bit, though, e.g., regarding color of the lines</t>
+  </si>
+  <si>
+    <t>Confirms</t>
+  </si>
+  <si>
+    <t>Results should not be affected too much by single observations.</t>
+  </si>
+  <si>
+    <t>Left observation Rauscher(2020) out</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>&lt;0.00000001</t>
+  </si>
+  <si>
+    <t>Inverse-variance WLS, cluster SE</t>
+  </si>
+  <si>
+    <t>Table 3, Column 1, Row 1</t>
+  </si>
+  <si>
+    <t>Table 4, Column 1, Row 1</t>
+  </si>
+  <si>
+    <t>Weakens</t>
+  </si>
+  <si>
+    <t>Results should not be affected too much by the selected method, in this case the random-effects meta-analysis method.</t>
+  </si>
+  <si>
+    <t>Summary
+This paper conducts a comprehensive meta-analysis of quasi-experimental studies examining the causal effects of US K–12 public school spending on student outcomes. The authors assemble a broad set of design-based estimates and study both average treatment effects and heterogeneity across contexts, populations, and policy environments. The paper’s central contribution is moving beyond the simple question of whether money matters toward estimating the distribution of likely policy effects across settings.
+The paper finds that increasing school spending by $1,000 per pupil for four years improves test scores by roughly 0.03 standard deviations and raises college-going rates by approximately 2.8 percentage points. The authors further argue that effects are relatively robust across geography and baseline spending levels, somewhat smaller for economically advantaged populations, and not substantially different between capital and noncapital expenditures. The paper also concludes that publication bias and confounding are limited.
+Design and Identification
+The paper’s design is strong overall. The authors appropriately restrict the meta-analysis to studies relying on quasi-random or quasi-experimental variation in school spending, which substantially improves the credibility of the underlying evidence base relative to older correlational literatures. The discussion of heterogeneity is also thoughtful and policy-relevant, especially given concerns about external validity in education research.
+The empirical framework is generally transparent and carefully implemented. The paper clearly explains study inclusion criteria, effect-size construction, and aggregation procedures. In addition, the discussion of uncertainty and treatment-effect heterogeneity is a major strength because it better reflects the range of plausible policy outcomes rather than presenting only a single pooled estimate.
+That said, several implementation and reproducibility details could be clarified further. While the authors provide replication materials, some coding choices reduce reproducibility for outside users. These issues do not appear to undermine the substantive conclusions, but addressing them would improve transparency and ease of replication.
+Robustness Checks
+I conducted two additional robustness checks.
+First, I assessed sensitivity to influential observations by removing the Rauscher (2020) estimate from the specification underlying Table 3. The main coefficient remained very similar in magnitude and statistical significance (original coefficient approximately 0.0316 versus robustness estimate approximately 0.0355). This suggests that the central findings are not being driven by a single influential study and strengthens confidence in the baseline result.
+Second, I re-estimated one specification using inverse-variance weighted least squares with clustered standard errors. Under this alternative weighting and inference procedure, the estimated coefficient became smaller and less statistically strong relative to the baseline specification. While the result still points in the same qualitative direction, the attenuation suggests that some conclusions may be somewhat sensitive to weighting assumptions and the treatment of uncertainty across studies. I do not view this as fatal, but I encourage the authors to discuss sensitivity to alternative meta-analytic weighting procedures more explicitly.
+Ethical and Transparency
+The replication package is overall well structured and easy to follow, which is a major strength of the paper. Providing a replication package at all is an important contribution to transparency and reproducibility. The code could, however, be made slightly more convenient to execute by defining key file paths globally, automatically creating required directories when needed, and documenting the package version numbers used in the analysis. These are relatively minor implementation improvements that would further enhance reproducibility without affecting the substantive findings.
+From an ethical and transparency perspective, the paper performs well in relying on publicly available administrative and study-level data rather than newly collected sensitive individual-level information. Since the paper is a meta-analysis, issues such as participant consent are primarily governed by the original studies included in the sample. While preregistration or registry information is not emphasized, the authors are transparent about their study-selection criteria, empirical procedures, and replication materials.
+Overall Assessment
+Overall, this is a strong and policy-relevant paper that makes a meaningful contribution to the literature on school spending and student outcomes. The empirical strategy is credible, the discussion of treatment-effect heterogeneity is particularly valuable, and the results appear broadly robust. Minor improvements to robustness discussion and replication convenience would further strengthen an already high-quality paper.</t>
   </si>
 </sst>
 </file>
@@ -923,21 +968,6 @@
   </cellStyleXfs>
   <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -979,11 +1009,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="19">
     <dxf>
       <fill>
         <patternFill>
@@ -1023,43 +1068,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFD1E7DD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF3F6FA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1408,82 +1416,82 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="9" width="26.5703125" style="6" customWidth="1"/>
+    <col min="1" max="9" width="26.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1502,116 +1510,116 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="26.5703125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="64.5703125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="30.5703125" style="6" customWidth="1"/>
-    <col min="7" max="7" width="22.5703125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="64.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="30.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
+      <c r="A4" s="1">
         <v>1</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="4">
         <v>46156.427083333336</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="6" t="s">
+    </row>
+    <row r="5" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>46156.447916666664</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" s="6">
-        <v>3</v>
-      </c>
-      <c r="B5" s="9">
-        <v>46156.447916666664</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4">
+        <v>46156.479166666664</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="E6" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
-        <v>4</v>
-      </c>
-      <c r="B6" s="9">
-        <v>46156.479166666664</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>84</v>
+      <c r="G6" s="1" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1619,28 +1627,28 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:G102">
-    <cfRule type="notContainsErrors" dxfId="22" priority="9">
+    <cfRule type="notContainsErrors" dxfId="18" priority="9">
       <formula>NOT(ISERROR(A4))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4:G103">
-    <cfRule type="expression" dxfId="21" priority="2">
+    <cfRule type="expression" dxfId="17" priority="2">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="3">
+    <cfRule type="expression" dxfId="16" priority="3">
       <formula>MOD(ROW(),2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:B103 D4:E103 G4:G103">
-    <cfRule type="expression" dxfId="19" priority="4">
+    <cfRule type="expression" dxfId="15" priority="4">
       <formula>LEN(TRIM(B4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:G1000">
-    <cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="Major">
+    <cfRule type="containsText" dxfId="14" priority="7" operator="containsText" text="Major">
       <formula>NOT(ISERROR(SEARCH("Major",G4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="8" operator="containsText" text="Minor">
+    <cfRule type="containsText" dxfId="13" priority="8" operator="containsText" text="Minor">
       <formula>NOT(ISERROR(SEARCH("Minor",G4)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1661,38 +1669,38 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.5703125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="60.5703125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="28.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="60.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="4">
+        <v>46156.493055555555</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="B3" s="9">
-        <v>46156.493055555555</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1700,45 +1708,27 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:A899">
-    <cfRule type="containsText" dxfId="16" priority="10" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="12" priority="10" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",A3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="11" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="11" priority="11" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",A3)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3">
-    <cfRule type="expression" dxfId="14" priority="9">
+  <conditionalFormatting sqref="A3:B3">
+    <cfRule type="expression" dxfId="10" priority="3">
       <formula>LEN(TRIM(A3))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3 C3">
-    <cfRule type="expression" dxfId="13" priority="6">
-      <formula>MOD(ROW(),2)=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="7">
-      <formula>MOD(ROW(),2)=1</formula>
-    </cfRule>
-    <cfRule type="notContainsErrors" dxfId="11" priority="8">
-      <formula>NOT(ISERROR(A3))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3">
-    <cfRule type="notContainsErrors" dxfId="10" priority="4">
-      <formula>NOT(ISERROR(B3))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3">
+  <conditionalFormatting sqref="A3:C3">
     <cfRule type="expression" dxfId="9" priority="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" dxfId="8" priority="2">
       <formula>MOD(ROW(),2)=1</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3">
-    <cfRule type="expression" dxfId="7" priority="3">
-      <formula>LEN(TRIM(B3))=0</formula>
+    <cfRule type="notContainsErrors" dxfId="7" priority="4">
+      <formula>NOT(ISERROR(A3))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -1758,127 +1748,186 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="26.5703125" style="6" customWidth="1"/>
-    <col min="5" max="8" width="20.5703125" style="11" customWidth="1"/>
-    <col min="9" max="13" width="26.5703125" style="6" customWidth="1"/>
-    <col min="14" max="17" width="20.5703125" style="11" customWidth="1"/>
-    <col min="18" max="18" width="26.5703125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="40" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+      <c r="P1" s="18"/>
+      <c r="Q1" s="18"/>
+      <c r="R1" s="18"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="3" t="s">
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
+      <c r="N2" s="20"/>
+      <c r="O2" s="20"/>
+      <c r="P2" s="20"/>
+      <c r="Q2" s="20"/>
+      <c r="R2" s="20"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="L3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="M3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="N3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="O3" s="8" t="s">
+      <c r="O3" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="P3" s="8" t="s">
+      <c r="P3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="Q3" s="8" t="s">
+      <c r="Q3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="R3" s="8" t="s">
+      <c r="R3" s="3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
+    <row r="4" spans="1:18" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4" s="1">
+        <v>3.1616720000000001E-2</v>
+      </c>
+      <c r="F4" s="1">
+        <v>2E-8</v>
+      </c>
+      <c r="G4" s="1">
+        <v>3.5456939999999999E-2</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="N4" s="1">
+        <v>3.2456435999999998E-2</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="P4" s="1">
+        <v>1.8833053999999998E-2</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>1.2915507999999999E-2</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1933,7 +1982,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
+    <col min="2" max="2" width="97.28515625" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
   </cols>
@@ -1942,7 +1991,7 @@
       <c r="A1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="7" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2016,7 +2065,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="8" t="s">
         <v>58</v>
       </c>
       <c r="B14" t="s">
@@ -2093,70 +2142,70 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
     </row>
     <row r="24" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
     </row>
     <row r="25" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="16"/>
+      <c r="A25" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="11"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="17"/>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="19"/>
+      <c r="A26" s="12"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="14"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="17"/>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="19"/>
+      <c r="A27" s="12"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="14"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="17"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="19"/>
+      <c r="A28" s="12"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="14"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="17"/>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="19"/>
+      <c r="A29" s="12"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="14"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="17"/>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="19"/>
+      <c r="A30" s="12"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="14"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="17"/>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="19"/>
+      <c r="A31" s="12"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="14"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="20"/>
-      <c r="B32" s="21"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="22"/>
+      <c r="A32" s="15"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
fix: changed numbering in Excel file
</commit_message>
<xml_diff>
--- a/report/Chris-Gabriel_Islam_Paper5_Replication_Log.xlsx
+++ b/report/Chris-Gabriel_Islam_Paper5_Replication_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Uni\Promotion\replication-game-kcl-2026\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A24BF0-1617-4161-B425-347C286DE9FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC71C04C-6631-405D-9CA7-3212FB0927BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Main" sheetId="1" r:id="rId1"/>
@@ -1009,6 +1009,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1017,12 +1023,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1420,17 +1420,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1520,15 +1520,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -1578,7 +1578,7 @@
     </row>
     <row r="5" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="4">
         <v>46156.447916666664</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="4">
         <v>46156.479166666664</v>
@@ -1675,11 +1675,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -1769,50 +1769,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="20" t="s">
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
-      <c r="O2" s="20"/>
-      <c r="P2" s="20"/>
-      <c r="Q2" s="20"/>
-      <c r="R2" s="20"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -2142,20 +2142,20 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
     </row>
     <row r="24" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="B24" s="22"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
     </row>
     <row r="25" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">

</xml_diff>